<commit_message>
Escala de stats, C6: registro de desvios, CLAUDE.md e a planilha com a escala aprovada
REGISTRO_DESVIOS: interpretações e desvios da Parte C (vida exibida sobre a
vida neutra, razão como fração exata, guts com o multiplicador, NPC neutro na
escala do estágio sugerido, só a campanha usa a escala, E4'/E4'' reprovados,
Sentinela sem fator que feche as metas, vários pets, tutorial). CLAUDE.md:
seção da planilha e da escala. A aba escala da planilha passa a ler a
ConfigEscala (CONFIG) e as taxas da validação (ARTEFATO): as 10 células SEM
FONTE da Parte B foram preenchidas; ficam as 5 da Parte A.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/artifacts_progressao/planilha_progressao.xlsx
+++ b/artifacts_progressao/planilha_progressao.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>fe81cab</t>
+          <t>a39b3d8</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T17:43:09-03:00</t>
+          <t>2026-09-28T18:28:33-03:00</t>
         </is>
       </c>
     </row>
@@ -8477,12 +8477,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>proposta (TAREFA B2: ~50 / 200 / 600 / 1500)</t>
-        </is>
-      </c>
-      <c r="J2" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.vida_por_estagio['bebe'] (aprovada na Parte B)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -8548,12 +8548,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>proposta (TAREFA B2: ~50 / 200 / 600 / 1500)</t>
-        </is>
-      </c>
-      <c r="J3" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.vida_por_estagio['crianca'] (aprovada na Parte B)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -8631,12 +8631,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>proposta (TAREFA B2: ~50 / 200 / 600 / 1500)</t>
-        </is>
-      </c>
-      <c r="J4" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.vida_por_estagio['adolescente'] (aprovada na Parte B)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -8714,12 +8714,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>proposta (TAREFA B2: ~50 / 200 / 600 / 1500)</t>
-        </is>
-      </c>
-      <c r="J5" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.vida_por_estagio['adulto'] (aprovada na Parte B)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -8930,12 +8930,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>proposta: 36 pontos → ×2,08 (o treino inteiro da vida pouco mais que dobra a escala)</t>
-        </is>
-      </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.beta_treino (36 pontos → ×2,08)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -8979,12 +8979,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>proposta: 36 pontos → ×2,08 (o treino inteiro da vida pouco mais que dobra a escala)</t>
-        </is>
-      </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.beta_treino (36 pontos → ×2,08)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -9028,12 +9028,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>proposta: 36 pontos → ×2,08 (o treino inteiro da vida pouco mais que dobra a escala)</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.beta_treino (36 pontos → ×2,08)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -9196,16 +9196,16 @@
         <v/>
       </c>
       <c r="D25" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>proposta: NPC na escala do estágio SUGERIDO para ele, um pouco acima do pet sem treino; calibrar na Parte C</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.fator_npc['tier1_brutamontes'] (calibrado: experiments/configs/escala/calibracao.json)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="G25" s="16">
@@ -9228,26 +9228,30 @@
         <f>(60+3.0*8)*0.6/(96*0.6)</f>
         <v/>
       </c>
-      <c r="L25" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr"/>
+      <c r="L25" t="n">
+        <v>0.2213</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier1_brutamontes.sem (sementes de validação)</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="O25" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr"/>
+          <t>ARTEFATO</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>0.9688</v>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier1_brutamontes.com</t>
+        </is>
+      </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
+          <t>ARTEFATO</t>
         </is>
       </c>
     </row>
@@ -9266,16 +9270,16 @@
         <v/>
       </c>
       <c r="D26" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>proposta: NPC na escala do estágio SUGERIDO para ele, um pouco acima do pet sem treino; calibrar na Parte C</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.fator_npc['tier2_sentinela'] (calibrado: experiments/configs/escala/calibracao.json)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="G26" s="16">
@@ -9298,26 +9302,30 @@
         <f>(60+3.0*22)*0.8/(72*1.0)</f>
         <v/>
       </c>
-      <c r="L26" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="L26" t="n">
+        <v>0.4125</v>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier2_sentinela.sem (sementes de validação)</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="O26" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr"/>
+          <t>ARTEFATO</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>0.7025</v>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier2_sentinela.com</t>
+        </is>
+      </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
+          <t>ARTEFATO</t>
         </is>
       </c>
     </row>
@@ -9336,16 +9344,16 @@
         <v/>
       </c>
       <c r="D27" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>proposta: NPC na escala do estágio SUGERIDO para ele, um pouco acima do pet sem treino; calibrar na Parte C</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.fator_npc['tier2_carcereiro'] (calibrado: experiments/configs/escala/calibracao.json)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="G27" s="16">
@@ -9368,26 +9376,30 @@
         <f>(60+3.0*22)*0.8/(90*1.0)</f>
         <v/>
       </c>
-      <c r="L27" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="L27" t="n">
+        <v>0.2606</v>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier2_carcereiro.sem (sementes de validação)</t>
+        </is>
+      </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="O27" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="P27" s="2" t="inlineStr"/>
+          <t>ARTEFATO</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>0.8413</v>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier2_carcereiro.com</t>
+        </is>
+      </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
+          <t>ARTEFATO</t>
         </is>
       </c>
     </row>
@@ -9406,16 +9418,16 @@
         <v/>
       </c>
       <c r="D28" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>proposta: NPC na escala do estágio SUGERIDO para ele, um pouco acima do pet sem treino; calibrar na Parte C</t>
-        </is>
-      </c>
-      <c r="F28" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.fator_npc['tier2_porteiro'] (calibrado: experiments/configs/escala/calibracao.json)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="G28" s="16">
@@ -9438,26 +9450,30 @@
         <f>(60+3.0*22)*0.8/(90*1.0)</f>
         <v/>
       </c>
-      <c r="L28" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="L28" t="n">
+        <v>0.1969</v>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier2_porteiro.sem (sementes de validação)</t>
+        </is>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="O28" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="P28" s="2" t="inlineStr"/>
+          <t>ARTEFATO</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>0.8938</v>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier2_porteiro.com</t>
+        </is>
+      </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
+          <t>ARTEFATO</t>
         </is>
       </c>
     </row>
@@ -9476,16 +9492,16 @@
         <v/>
       </c>
       <c r="D29" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>proposta: NPC na escala do estágio SUGERIDO para ele, um pouco acima do pet sem treino; calibrar na Parte C</t>
-        </is>
-      </c>
-      <c r="F29" s="10" t="inlineStr">
-        <is>
-          <t>PROPOSTO</t>
+          <t>digilab/config.py &gt; ConfigEscala.fator_npc['tier3_soberano'] (calibrado: experiments/configs/escala/calibracao.json)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CONFIG</t>
         </is>
       </c>
       <c r="G29" s="16">
@@ -9508,26 +9524,30 @@
         <f>(60+3.0*36)*1.0/(110*1.0)</f>
         <v/>
       </c>
-      <c r="L29" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="L29" t="n">
+        <v>0.1688</v>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier3_soberano.sem (sementes de validação)</t>
+        </is>
+      </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="O29" s="14" t="inlineStr">
-        <is>
-          <t>SEM FONTE</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="inlineStr"/>
+          <t>ARTEFATO</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>0.9116</v>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>experiments/configs/escala/validacao.json &gt; resultado.tier3_soberano.com</t>
+        </is>
+      </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>SEM FONTE</t>
+          <t>ARTEFATO</t>
         </is>
       </c>
     </row>
@@ -9539,7 +9559,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>com os fatores propostos a razão pet/NPC fica abaixo de 1,0 sem treino e acima com o treino típico em todos os portões (Brutamontes (Gazimon) 0,87 → 1,08; Sentinela (Tortomon) 0,83 → 1,38; Carcereiro 0,77 → 1,28; Porteiro 0,77 → 1,28; Soberano 0,62 → 1,30). Os NPCs da Torre deixam de ter tamanho de adulto: passam à escala do Champion. A taxa esperada só existe depois de rodar (Parte C: calibrar_progressao nas sementes de calibração). As razões de hoje usam o modelo de poder da aba jornada (contas sobre os valores do config.py, visíveis na fórmula).</t>
+          <t>com os fatores propostos a razão pet/NPC fica abaixo de 1,0 sem treino e acima com o treino típico em todos os portões (Brutamontes (Gazimon) 0,91 → 1,13; Sentinela (Tortomon) 0,62 → 1,04; Carcereiro 0,67 → 1,11; Porteiro 0,91 → 1,51; Soberano 0,83 → 1,73). Os NPCs da Torre deixam de ter tamanho de adulto: passam à escala do Champion. As taxas vêm da validação da Parte C (experiments/calibrar_escala.py --validar); a Sentinela não fecha com nenhum fator (estilo tartaruga). As razões de hoje usam o modelo de poder da aba jornada (contas sobre os valores do config.py, visíveis na fórmula).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Escala: exceção da Sentinela aceita e E4 redefinido (decisões do Matheus)
E4 na escala: a evolução sempre importa. O adulto sem treino vence o
adolescente da mesma linha, sem treino e com o treino máximo do estágio (+22),
em ≥ 0,60, sem teto (ConfigEscala.taxa_min_e4; gate E4_escala_estagio_importa).
Sai o E4' (faixa [0,60, 0,85]) e o E4'' (≥ 0,90) da Parte B.

Bateria V21C com a escala rodada de novo (artifacts_combate_v21c/
validacao_escala): E4 passa (menor 0,836); E1, E3, E5 (25/36), guardião, G9,
base V2C e sanidade iguais; E2, G6b e G8 seguem como exceções aceitas.
Sentinela: exceção aceita (fator 1,6; 0,41 → 0,70 na validação). Registro de
desvios, CLAUDE.md, JORNADA_JOGADOR.md e a aba escala da planilha atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/artifacts_progressao/planilha_progressao.xlsx
+++ b/artifacts_progressao/planilha_progressao.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>a39b3d8</t>
+          <t>8414ab6</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T18:28:33-03:00</t>
+          <t>2026-09-28T18:29:32-03:00</t>
         </is>
       </c>
     </row>
@@ -9566,7 +9566,7 @@
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>E4 redefinido (B2.6, PROPOSTO)</t>
+          <t>E4 redefinido (B2.6; definição final do Matheus depois da Parte C)</t>
         </is>
       </c>
     </row>
@@ -9578,12 +9578,12 @@
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>hoje</t>
+          <t>antes da escala</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>proposta</t>
+          <t>na escala</t>
         </is>
       </c>
     </row>
@@ -9600,7 +9600,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>o treino fecha parte da distância entre estágios: adulto SEM treino × adolescente com o treino MÁXIMO do estágio (22 pontos)</t>
+          <t>a evolução sempre importa: adulto SEM treino × adolescente sem treino e com o treino máximo do estágio (+22)</t>
         </is>
       </c>
     </row>
@@ -9617,7 +9617,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>taxa do adulto em [0,60, 0,85] com o adolescente treinado; e adulto sem treino × adolescente sem treino ≥ 0,90 (o 'stat check' é de propósito)</t>
+          <t>taxa do adulto ≥ 0,60 nos dois casos, sem teto (esmagar é de propósito na escala)</t>
         </is>
       </c>
     </row>
@@ -9629,19 +9629,19 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>com escala de franquia o adulto sem treino esmaga o adolescente sem treino (E_adulto/E_adol = 2,5)</t>
+          <t>com escala de franquia o adulto sem treino esmaga o adolescente (E_adulto/E_Champion = 2,5)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>a pergunta vira 'o treino do estágio anterior compensa um pouco a evolução?' (princípio 7: treinar cedo rende)</t>
+          <t>a Parte B propunha E4' (treino compensa: faixa [0,60, 0,85]) e E4'' (≥ 0,90); os dois reprovaram e o Matheus redefiniu</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>resultado de hoje</t>
+          <t>resultado</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>SEM FONTE até a Parte C (bateria V21C com a escala ligada)</t>
+          <t>OK — adulto sem treino x adolescente (sem treino e com +22): abaixo de 0.6: nenhum; menor 0.836</t>
         </is>
       </c>
     </row>

</xml_diff>